<commit_message>
Sửa kiện OM4-DE-IS-0009-005 qua web
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,6 +416,15 @@
       <c r="E1" t="str">
         <v>Vị trí</v>
       </c>
+      <c r="F1" t="str">
+        <v>Trạng thái</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Ngày xuất</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Ngày cập nhật</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -431,12 +440,21 @@
         <v>OM4-DE-IS-0009</v>
       </c>
       <c r="E2" t="str">
-        <v>Y3-4</v>
+        <v>Y3-1</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>18/08/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sửa theo P/L OM4-DE-IS-0009 (17 kiện) qua web
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -452,9 +452,425 @@
         <v>18/08/2026</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>OM4-DE-IS-0009-001</v>
+      </c>
+      <c r="C3" t="str">
+        <v>HDG STEEL Conduit</v>
+      </c>
+      <c r="D3" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>OM4-DE-IS-0009-002</v>
+      </c>
+      <c r="C4" t="str">
+        <v>HDG STEEL Conduit</v>
+      </c>
+      <c r="D4" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>OM4-DE-IS-0009-003</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CONDUIT FITTINGS</v>
+      </c>
+      <c r="D5" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>OM4-DE-IS-0009-004</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CONDUIT FITTINGS (Normal Bend)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>OM4-DE-IS-0009-006</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CONDUIT FITTINGS (Normal Bend)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>OM4-DE-IS-0009-007</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CONDUIT FITTINGS (Normal Bend)</v>
+      </c>
+      <c r="D8" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>OM4-DE-IS-0009-008</v>
+      </c>
+      <c r="C9" t="str">
+        <v>CONDUIT FITTINGS (Normal Bend)</v>
+      </c>
+      <c r="D9" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>OM4-DE-IS-0009-009</v>
+      </c>
+      <c r="C10" t="str">
+        <v>CONDUIT FITTINGS (Normal Bend)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>OM4-DE-IS-0009-010</v>
+      </c>
+      <c r="C11" t="str">
+        <v>CONDUIT FITTINGS</v>
+      </c>
+      <c r="D11" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>OM4-DE-IS-0009-011</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Flexible Conduit</v>
+      </c>
+      <c r="D12" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>OM4-DE-IS-0009-012</v>
+      </c>
+      <c r="C13" t="str">
+        <v>CONDUIT FITTINGS</v>
+      </c>
+      <c r="D13" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>OM4-DE-IS-0009-013</v>
+      </c>
+      <c r="C14" t="str">
+        <v>PULL BOX with C-COVER</v>
+      </c>
+      <c r="D14" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>OM4-DE-IS-0009-014</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Post Base single Channel</v>
+      </c>
+      <c r="D15" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>OM4-DE-IS-0009-015</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Unistrut Channel Single</v>
+      </c>
+      <c r="D16" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>OM4-DE-IS-0009-016</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Uni-Struct Insert channel</v>
+      </c>
+      <c r="D17" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>28/07/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>OM4-DE-IS-0009-017</v>
+      </c>
+      <c r="C18" t="str">
+        <v>C- Channel</v>
+      </c>
+      <c r="D18" t="str">
+        <v>OM4-DE-IS-0009</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Y3-2</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sửa kiện OM4-P2-LS-0002-001 qua web
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -868,9 +868,35 @@
         <v>18/08/2026</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>OM4-P2-LS-0002-001</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Stranded Bare Copper Conductor 240 sq.mm(C-240)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>OM4-P2-LS-0002</v>
+      </c>
+      <c r="E19" t="str">
+        <v>S1</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v>18/08/2026</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Xuất 1 PKG HRSG Embeded Material - kiện OM4-DE-IS-0002-002
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -413,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -572,12 +572,92 @@
         <v/>
       </c>
       <c r="Z2" t="str">
-        <v>[{"name":"HRSG Embeded Material (Template)","qty":1,"unit":"PKG","remaining":1,"log":[{"time":"21:59:36 18/8/2026","change":1,"after":1},{"time":"21:59:33 18/8/2026","change":-1,"after":0}]},{"name":"TEMPLATE(TP-1)_10T*374*374","qty":20,"unit":"EA","remaining":18,"log":[{"time":"22:05:53 18/8/2026","change":-1,"after":18},{"time":"22:00:37 18/8/2026","change":-1,"after":19}]},{"name":"TEMPLATE(TP-2)_10T*450*900","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"TEMPLATE(TP-3)_10T*270*320","qty":8,"unit":"EA","remaining":8,"log":[]},{"name":"TEMPLATE(STP-1)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-2)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-3)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-4)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]}]</v>
+        <v>[{"name":"HRSG Embeded Material (Template)","qty":1,"unit":"PKG","remaining":1,"log":[{"time":"21:59:36 18/8/2026","change":1,"after":1},{"time":"21:59:33 18/8/2026","change":-1,"after":0}]},{"name":"TEMPLATE(TP-1)_10T*374*374","qty":20,"unit":"EA","remaining":19,"log":[{"time":"22:00:37 18/8/2026","change":-1,"after":19}]},{"name":"TEMPLATE(TP-2)_10T*450*900","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"TEMPLATE(TP-3)_10T*270*320","qty":8,"unit":"EA","remaining":8,"log":[]},{"name":"TEMPLATE(STP-1)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-2)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-3)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-4)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]}]</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>OM4-DE-IS-0002-002</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v>[{"name":"HRSG Embeded Material","qty":1,"unit":"PKG","remaining":0,"log":[{"time":"22:07:45 18/8/2026","change":-1,"after":0}]},{"name":"Anchor Bolt M56X1,515L","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Nut M56","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Anchor Bolt M42X1,110L","qty":16,"unit":"EA","remaining":16,"log":[]},{"name":"Nut M42","qty":64,"unit":"EA","remaining":64,"log":[]}]</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nhập trả 1 EA TEMPLATE(TP-1)_10T*374*374 - kiện OM4-DE-IS-0001-001
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -413,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:Z2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -572,92 +572,12 @@
         <v/>
       </c>
       <c r="Z2" t="str">
-        <v>[{"name":"HRSG Embeded Material (Template)","qty":1,"unit":"PKG","remaining":1,"log":[{"time":"21:59:36 18/8/2026","change":1,"after":1},{"time":"21:59:33 18/8/2026","change":-1,"after":0}]},{"name":"TEMPLATE(TP-1)_10T*374*374","qty":20,"unit":"EA","remaining":19,"log":[{"time":"22:00:37 18/8/2026","change":-1,"after":19}]},{"name":"TEMPLATE(TP-2)_10T*450*900","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"TEMPLATE(TP-3)_10T*270*320","qty":8,"unit":"EA","remaining":8,"log":[]},{"name":"TEMPLATE(STP-1)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-2)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-3)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-4)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]}]</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>18/08/2026</v>
-      </c>
-      <c r="B3" t="str">
-        <v>OM4-DE-IS-0002-002</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v>Trong kho</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>18/08/2026</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
-      <c r="R3" t="str">
-        <v/>
-      </c>
-      <c r="S3" t="str">
-        <v/>
-      </c>
-      <c r="T3" t="str">
-        <v/>
-      </c>
-      <c r="U3" t="str">
-        <v/>
-      </c>
-      <c r="V3" t="str">
-        <v/>
-      </c>
-      <c r="W3" t="str">
-        <v/>
-      </c>
-      <c r="X3" t="str">
-        <v/>
-      </c>
-      <c r="Y3" t="str">
-        <v/>
-      </c>
-      <c r="Z3" t="str">
-        <v>[{"name":"HRSG Embeded Material","qty":1,"unit":"PKG","remaining":0,"log":[{"time":"22:07:45 18/8/2026","change":-1,"after":0}]},{"name":"Anchor Bolt M56X1,515L","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Nut M56","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Anchor Bolt M42X1,110L","qty":16,"unit":"EA","remaining":16,"log":[]},{"name":"Nut M42","qty":64,"unit":"EA","remaining":64,"log":[]}]</v>
+        <v>[{"name":"HRSG Embeded Material (Template)","qty":1,"unit":"PKG","remaining":1,"log":[{"time":"21:59:36 18/8/2026","change":1,"after":1},{"time":"21:59:33 18/8/2026","change":-1,"after":0}]},{"name":"TEMPLATE(TP-1)_10T*374*374","qty":20,"unit":"EA","remaining":20,"log":[{"time":"22:09:54 18/8/2026","change":1,"after":20},{"time":"22:00:37 18/8/2026","change":-1,"after":19}]},{"name":"TEMPLATE(TP-2)_10T*450*900","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"TEMPLATE(TP-3)_10T*270*320","qty":8,"unit":"EA","remaining":8,"log":[]},{"name":"TEMPLATE(STP-1)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-2)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-3)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-4)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]}]</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Xuất 1 PKG HRSG Embeded Material (Anchor Bolt/Nut/Washer) - kiện OM4-DE-IS-0001-002
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -413,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -575,9 +575,89 @@
         <v>[{"name":"HRSG Embeded Material (Template)","qty":1,"unit":"PKG","remaining":1,"log":[{"time":"21:59:36 18/8/2026","change":1,"after":1},{"time":"21:59:33 18/8/2026","change":-1,"after":0}]},{"name":"TEMPLATE(TP-1)_10T*374*374","qty":20,"unit":"EA","remaining":20,"log":[{"time":"22:09:54 18/8/2026","change":1,"after":20},{"time":"22:00:37 18/8/2026","change":-1,"after":19}]},{"name":"TEMPLATE(TP-2)_10T*450*900","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"TEMPLATE(TP-3)_10T*270*320","qty":8,"unit":"EA","remaining":8,"log":[]},{"name":"TEMPLATE(STP-1)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-2)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-3)_15T*250*3801","qty":6,"unit":"EA","remaining":6,"log":[]},{"name":"TEMPLATE(STP-4)_10T*60*250","qty":6,"unit":"EA","remaining":6,"log":[]}]</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>OM4-DE-IS-0001-002</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v>[{"name":"HRSG Embeded Material (Anchor Bolt/Nut/Washer)","qty":1,"unit":"PKG","remaining":0,"log":[{"time":"22:18:37 18/8/2026","change":-1,"after":0}]},{"name":"Anchor Bolt","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Nut M56","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Anchor Bolt","qty":16,"unit":"EA","remaining":16,"log":[]},{"name":"Nut M42","qty":64,"unit":"EA","remaining":64,"log":[]}]</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Xuất 1 EA Bot. Plate 100X100X10T - kiện OM4-DE-IS-0001-007
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -580,7 +580,7 @@
         <v>18/08/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>OM4-DE-IS-0001-002</v>
+        <v>OM4-DE-IS-0001-007</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -652,7 +652,7 @@
         <v/>
       </c>
       <c r="Z3" t="str">
-        <v>[{"name":"HRSG Embeded Material (Anchor Bolt/Nut/Washer)","qty":1,"unit":"PKG","remaining":1,"log":[{"time":"22:18:42 18/8/2026","change":1,"after":1},{"time":"22:18:37 18/8/2026","change":-1,"after":0}]},{"name":"Anchor Bolt","qty":40,"unit":"EA","remaining":40,"log":[{"time":"22:18:56 18/8/2026","change":1,"after":40},{"time":"22:18:44 18/8/2026","change":-1,"after":39}]},{"name":"Nut M56","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Anchor Bolt","qty":16,"unit":"EA","remaining":16,"log":[]},{"name":"Nut M42","qty":64,"unit":"EA","remaining":64,"log":[]}]</v>
+        <v>[{"name":"HRSG Embeded Material (Anchor Bolt/Nut/Washer)","qty":1,"unit":"PKG","remaining":1,"log":[]},{"name":"Square Washer 130X160X20T","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Square Washer 130X130X20T","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Square Washer 100X100X15T","qty":16,"unit":"EA","remaining":16,"log":[]},{"name":"Square Washer 120X120X16T","qty":72,"unit":"EA","remaining":72,"log":[]},{"name":"Anchor Plate 130X130X20T","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Anchor Plate 130X130X20T","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Anchor Plate 100X100X12T","qty":16,"unit":"EA","remaining":16,"log":[]},{"name":"Anchor Plate 120X120X16T","qty":72,"unit":"EA","remaining":72,"log":[]},{"name":"Bot. Plate 100X100X10T","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Bot. Plate 100X100X10T","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Bot. Plate 100X100X10T","qty":16,"unit":"EA","remaining":15,"log":[{"time":"22:19:49 18/8/2026","change":-1,"after":15}]}]</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Xuất 1 EA Condulet ("LT" Type) 28mm (1") - kiện OM4-DE-IS-0009-010
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -413,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:Z4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -655,9 +655,89 @@
         <v>[{"name":"HRSG Embeded Material (Anchor Bolt/Nut/Washer)","qty":1,"unit":"PKG","remaining":1,"log":[]},{"name":"Square Washer 130X160X20T","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Square Washer 130X130X20T","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Square Washer 100X100X15T","qty":16,"unit":"EA","remaining":16,"log":[]},{"name":"Square Washer 120X120X16T","qty":72,"unit":"EA","remaining":72,"log":[]},{"name":"Anchor Plate 130X130X20T","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Anchor Plate 130X130X20T","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Anchor Plate 100X100X12T","qty":16,"unit":"EA","remaining":16,"log":[]},{"name":"Anchor Plate 120X120X16T","qty":72,"unit":"EA","remaining":72,"log":[]},{"name":"Bot. Plate 100X100X10T","qty":40,"unit":"EA","remaining":40,"log":[]},{"name":"Bot. Plate 100X100X10T","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Bot. Plate 100X100X10T","qty":16,"unit":"EA","remaining":16,"log":[{"time":"22:19:52 18/8/2026","change":1,"after":16},{"time":"22:19:49 18/8/2026","change":-1,"after":15}]}]</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>OM4-DE-IS-0009-010</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>18/08/2026</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v>[{"name":"Condulet (\"LT\" Type) 28mm (1\")","qty":30,"unit":"EA","remaining":29,"log":[{"time":"22:30:41 18/8/2026","change":-1,"after":29}]},{"name":"Condulet (\"LT\" Type) 36mm (1-1/4\")","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"Condulet (\"LT\" Type) 42mm (1-1/2\")","qty":10,"unit":"EA","remaining":10,"log":[]},{"name":"Condulet (\"LT\" Type) 54mm (2\")","qty":15,"unit":"EA","remaining":15,"log":[]},{"name":"Condulet (\"LT\" Type) 82mm (3\")","qty":15,"unit":"EA","remaining":15,"log":[]},{"name":"Condulet (\"LT\" Type) 104mm (4\")","qty":10,"unit":"EA","remaining":10,"log":[]},{"name":"Flexible Conduit Connector (Male Type) 28mm (1\")","qty":420,"unit":"EA","remaining":420,"log":[]},{"name":"Flexible Conduit Connector (Male Type) 36mm (1-1/4\")","qty":150,"unit":"EA","remaining":150,"log":[]},{"name":"Flexible Conduit Connector (Male Type) 42mm (1-1/2\")","qty":50,"unit":"EA","remaining":50,"log":[]},{"name":"Flexible Conduit Connector (Male Type) 54mm (2\")","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"Flexible Conduit Connector (Male Type) 82mm (3\")","qty":80,"unit":"EA","remaining":80,"log":[]},{"name":"Flexible Conduit Connector (Male Type) 104mm (4\")","qty":50,"unit":"EA","remaining":50,"log":[]},{"name":"Flexible Conduit Connector (Female Type) 28mm (1\")","qty":420,"unit":"EA","remaining":420,"log":[]},{"name":"Flexible Conduit Connector (Female Type) 36mm (1-1/4\")","qty":150,"unit":"EA","remaining":150,"log":[]},{"name":"Flexible Conduit Connector (Female Type) 42mm (1-1/2\")","qty":50,"unit":"EA","remaining":50,"log":[]},{"name":"Flexible Conduit Connector (Female Type) 54mm (2\")","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"Flexible Conduit Connector (Female Type) 82mm (3\")","qty":80,"unit":"EA","remaining":80,"log":[]},{"name":"Flexible Conduit Connector (Female Type) 104mm (4\")","qty":50,"unit":"EA","remaining":50,"log":[]},{"name":"Union Coupling (Male Type) 28mm (1\")","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"Union Coupling (Male Type) 36mm (1-1/4\")","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"Union Coupling (Male Type) 42mm (1-1/2\")","qty":10,"unit":"EA","remaining":10,"log":[]},{"name":"Union Coupling (Male Type) 54mm (2\")","qty":10,"unit":"EA","remaining":10,"log":[]},{"name":"Union Coupling (Male Type) 82mm (3\")","qty":10,"unit":"EA","remaining":10,"log":[]},{"name":"Nipple(EXPLOSION TYPE, NPT to PF) 28mm (1\")","qty":10,"unit":"EA","remaining":10,"log":[]},{"name":"Nipple(EXPLOSION TYPE, NPT to PF) 36mm (1-1/4\")","qty":5,"unit":"EA","remaining":5,"log":[]},{"name":"Nipple(EXPLOSION TYPE, NPT to PF) 42mm (1-1/2\")","qty":5,"unit":"EA","remaining":5,"log":[]},{"name":"Nipple(EXPLOSION TYPE, NPT to PF) 54mm (2\")","qty":5,"unit":"EA","remaining":5,"log":[]},{"name":"SEALING COMPOUND Plaster FOR SEALING FITTING 1KG/CAN","qty":50,"unit":"EA","remaining":50,"log":[]},{"name":"REDUCER(ADAPTER TYPE) 36mm Male - 28mm Female","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"REDUCER(ADAPTER TYPE) 36mm Male - 28mm Female","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"REDUCER(ADAPTER TYPE) 42mm Male - 28mm Female","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"REDUCER(ADAPTER TYPE) 54mm Male - 28mm Female","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"REDUCER(ADAPTER TYPE) 54mm Male - 42mm Female","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"REDUCER(ADAPTER TYPE) 28mm Male - 42mm Female","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"REDUCER(ADAPTER TYPE) 36mm Male - 28mm Female","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"REDUCER(ADAPTER TYPE) 42mm Male - 36mm Female","qty":30,"unit":"EA","remaining":30,"log":[]},{"name":"Lock Nut 28mm (1\")","qty":800,"unit":"EA","remaining":800,"log":[]},{"name":"Lock Nut 36mm (1-1/4\")","qty":200,"unit":"EA","remaining":200,"log":[]},{"name":"Lock Nut 42mm (1-1/2\")","qty":100,"unit":"EA","remaining":100,"log":[]},{"name":"Lock Nut 54mm (2\")","qty":50,"unit":"EA","remaining":50,"log":[]},{"name":"Lock Nut 82mm (3\")","qty":160,"unit":"EA","remaining":160,"log":[]},{"name":"Lock Nut 104mm (4\")","qty":100,"unit":"EA","remaining":100,"log":[]},{"name":"Lock Nut 125mm (5\")","qty":120,"unit":"EA","remaining":120,"log":[]},{"name":"Flexible Conduit (Water proof type) 36mm (1-1/4\")","qty":330,"unit":"M","remaining":330,"log":[]}]</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sửa theo P/L OM4-DE-IS-0011 (2 kiện) qua web
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -568,9 +568,169 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>OM4-DE-IS-0011-001</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Coupling for Steel Conduit 125mm (5") (50 EA); Flexible Conduit Connector (Male Type) 125mm (5") (50 EA); Flexible Conduit Connector (Female Type) 125mm (5") (50 EA); PIPE CLAMP With Bolt/Nut/Washer 125mm (5") (500 SET); Insulation Bushing W/Earthing 150mm (6") (70 EA)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>OM4-DE-IS-0011</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Office</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>OM4-DE-IS-0011-002</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Flexible Conduit (Water proof type) 125mm (5") (120 M)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>OM4-DE-IS-0011</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Office</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Đổi vị trí hàng loạt (1 kiện) qua web
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:Z5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -502,7 +502,7 @@
         <v>OM4-DE-IS-0001</v>
       </c>
       <c r="E2" t="str">
-        <v>S1</v>
+        <v/>
       </c>
       <c r="F2" t="str">
         <v>Trong kho</v>
@@ -728,9 +728,89 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>OM4-DE-IS-0001-002</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Anchor Bolt (40 EA); Nut M56 (160 EA); Anchor Bolt (16 EA); Nut M42 (64 EA)</v>
+      </c>
+      <c r="D5" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E5" t="str">
+        <v>S2</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sửa theo P/L OM4-DE-IS-0001 (10 kiện) qua web
</commit_message>
<xml_diff>
--- a/du-lieu/chinh-sua-tay.xlsx
+++ b/du-lieu/chinh-sua-tay.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z5"/>
+  <dimension ref="A1:Z13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -502,7 +502,7 @@
         <v>OM4-DE-IS-0001</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>S3</v>
       </c>
       <c r="F2" t="str">
         <v>Trong kho</v>
@@ -742,7 +742,7 @@
         <v>OM4-DE-IS-0001</v>
       </c>
       <c r="E5" t="str">
-        <v>S2</v>
+        <v>S3</v>
       </c>
       <c r="F5" t="str">
         <v>Trong kho</v>
@@ -805,12 +805,652 @@
         <v/>
       </c>
       <c r="Z5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>OM4-DE-IS-0001-003</v>
+      </c>
+      <c r="C6" t="str">
+        <v>HRSG Embeded Material (Anchor Bolt/Nut/Washer) (1 PKG); Anchor Bolt (53 EA); Nut M60 (212 EA)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E6" t="str">
+        <v>S3</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>OM4-DE-IS-0001-004</v>
+      </c>
+      <c r="C7" t="str">
+        <v>HRSG Embeded Material (Anchor Bolt/Nut/Washer) (1 PKG); Anchor Bolt (53 EA); Nut M60 (212 EA)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E7" t="str">
+        <v>S3</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>OM4-DE-IS-0001-005</v>
+      </c>
+      <c r="C8" t="str">
+        <v>HRSG Embeded Material (Anchor Bolt/Nut/Washer) (1 PKG); Anchor Bolt (54 EA); Nut M60 (216 EA)</v>
+      </c>
+      <c r="D8" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E8" t="str">
+        <v>S3</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>OM4-DE-IS-0001-006</v>
+      </c>
+      <c r="C9" t="str">
+        <v>HRSG Embeded Material (Anchor Bolt/Nut/Washer) (1 PKG); Anchor Bolt (72 EA); Nut M48 (288 EA)</v>
+      </c>
+      <c r="D9" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E9" t="str">
+        <v>S3</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>OM4-DE-IS-0001-007</v>
+      </c>
+      <c r="C10" t="str">
+        <v>HRSG Embeded Material (Anchor Bolt/Nut/Washer) (1 PKG); Square Washer 130X160X20T (40 EA); Square Washer 130X130X20T (160 EA); Square Washer 100X100X15T (16 EA); Square Washer 120X120X16T (72 EA); Anchor Plate 130X130X20T (40 EA); Anchor Plate 130X130X20T (160 EA); Anchor Plate 100X100X12T (16 EA); Anchor Plate 120X120X16T (72 EA); Bot. Plate 100X100X10T (40 EA); Bot. Plate 100X100X10T (160 EA); Bot. Plate 100X100X10T (16 EA)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E10" t="str">
+        <v>S3</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>OM4-DE-IS-0001-008</v>
+      </c>
+      <c r="C11" t="str">
+        <v>HRSG Embeded Material (Anchor Bolt/Nut/Washer) (1 PKG); Sleeve 3"XSTD-982L (40 EA); Sleeve 3"XSTD-1,062L (160 EA); Sleeve 2-1/2"XSTD-752L (16 EA); Cap Plate Ø100XØ61X10T (40 EA); Cap Plate Ø100XØ65X10T (160 EA); Cap Plate Ø100XØ47X10T (16 EA)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E11" t="str">
+        <v>S3</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>OM4-DE-IS-0001-009</v>
+      </c>
+      <c r="C12" t="str">
+        <v>HRSG Embeded Material (Spare) (1 PKG); Nut M56 (8 EA); Nut M60 (32 EA); Nut M42 (5 EA); Nut M48 (14 EA); Square Washer 130X160X20T (5 EA); Square Washer 130X130X20T (8 EA); Square Washer 100X100X15T (5 EA); Square Washer 120X120X16T (5 EA)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E12" t="str">
+        <v>S3</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
+        <v/>
+      </c>
+      <c r="Z12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>S1</v>
+      </c>
+      <c r="C13" t="str">
+        <v>HRSG Embeded Material (Template)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>OM4-DE-IS-0001</v>
+      </c>
+      <c r="E13" t="str">
+        <v>S3</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Trong kho</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v>19/08/2026</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v/>
+      </c>
+      <c r="Z13" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>